<commit_message>
delte files unused in 4.0.5, run full csv exporter
</commit_message>
<xml_diff>
--- a/InputData/ccs/CC/CCS Calculations.xlsx
+++ b/InputData/ccs/CC/CCS Calculations.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28317"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26827"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -54,20 +54,14 @@
     <definedName name="solver_val" localSheetId="0" hidden="1">0.15</definedName>
     <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -77,6 +71,216 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="98">
   <si>
+    <t>Source:</t>
+  </si>
+  <si>
+    <t>Notes:</t>
+  </si>
+  <si>
+    <t>Capital cost ($/(metric ton CO2e*yr))</t>
+  </si>
+  <si>
+    <t>O&amp;M Cost per Ton ($/metric ton CO2e)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This variable captures the capital and O&amp;M costs and energy use of </t>
+  </si>
+  <si>
+    <t>The energy use value here should exclude any energy that is not additional</t>
+  </si>
+  <si>
+    <t>isn't being used, and they use it to power CCS, that heat should be excluded</t>
+  </si>
+  <si>
+    <t>from here, since it does not increase the overall energy demand of the steel</t>
+  </si>
+  <si>
+    <t>mill.</t>
+  </si>
+  <si>
+    <t>agriculture and forestry 01T03</t>
+  </si>
+  <si>
+    <t>coal mining 05</t>
+  </si>
+  <si>
+    <t>oil and gas extraction 06</t>
+  </si>
+  <si>
+    <t>other mining and quarrying 07T08</t>
+  </si>
+  <si>
+    <t>food beverage and tobacco 10T12</t>
+  </si>
+  <si>
+    <t>textiles apparel and leather 13T15</t>
+  </si>
+  <si>
+    <t>wood products 16</t>
+  </si>
+  <si>
+    <t>pulp paper and printing 17T18</t>
+  </si>
+  <si>
+    <t>refined petroleum and coke 19</t>
+  </si>
+  <si>
+    <t>chemicals 20</t>
+  </si>
+  <si>
+    <t>rubber and plastic products 22</t>
+  </si>
+  <si>
+    <t>glass and glass products 231</t>
+  </si>
+  <si>
+    <t>cement and other nonmetallic minerals 239</t>
+  </si>
+  <si>
+    <t>iron and steel 241</t>
+  </si>
+  <si>
+    <t>other metals 242</t>
+  </si>
+  <si>
+    <t>metal products except machinery and vehicles 25</t>
+  </si>
+  <si>
+    <t>computers and electronics 26</t>
+  </si>
+  <si>
+    <t>appliances and electrical equipment 27</t>
+  </si>
+  <si>
+    <t>other machinery 28</t>
+  </si>
+  <si>
+    <t>road vehicles 29</t>
+  </si>
+  <si>
+    <t>nonroad vehicles 30</t>
+  </si>
+  <si>
+    <t>other manufacturing 31T33</t>
+  </si>
+  <si>
+    <t>energy pipelines and gas processing 352T353</t>
+  </si>
+  <si>
+    <t>water and waste 36T39</t>
+  </si>
+  <si>
+    <t>construction 41T43</t>
+  </si>
+  <si>
+    <t>Gaffney Cline</t>
+  </si>
+  <si>
+    <t>National Petroleum Council (NPC) Capture Facility Reference Costs</t>
+  </si>
+  <si>
+    <t>https://www.gaffneycline.com/calculator/npc-scenarios-table</t>
+  </si>
+  <si>
+    <t>Facility Type</t>
+  </si>
+  <si>
+    <t>Low Estimates</t>
+  </si>
+  <si>
+    <t>Capacity (tonne / year)</t>
+  </si>
+  <si>
+    <t>Total CapEx (US $ / annual tonne)</t>
+  </si>
+  <si>
+    <t>Natural Gas Processing</t>
+  </si>
+  <si>
+    <t>Electricity usage (MWh / tonne)</t>
+  </si>
+  <si>
+    <t>Gas usage (MWh / tonne)</t>
+  </si>
+  <si>
+    <t>OpEx, Non-energy, annual (% CapEx)</t>
+  </si>
+  <si>
+    <t>Tax rate (%)</t>
+  </si>
+  <si>
+    <t>High Estimates</t>
+  </si>
+  <si>
+    <t>Averages</t>
+  </si>
+  <si>
+    <t>CapEx ($ / annual tonne)</t>
+  </si>
+  <si>
+    <t>Electricity usage (BTU / tonne)</t>
+  </si>
+  <si>
+    <t>Gas usage (BTU / tonne)</t>
+  </si>
+  <si>
+    <t>OpEx, Non-energy</t>
+  </si>
+  <si>
+    <t>BTU per MWh</t>
+  </si>
+  <si>
+    <t>Ethanol Production</t>
+  </si>
+  <si>
+    <t>Ammonia Production</t>
+  </si>
+  <si>
+    <t>Hydrogen Production</t>
+  </si>
+  <si>
+    <t>Cement Plant</t>
+  </si>
+  <si>
+    <t>Refinery Fluidized Catalytic Converter</t>
+  </si>
+  <si>
+    <t>Iron and Steel Plant</t>
+  </si>
+  <si>
+    <t>Industrial Furnace</t>
+  </si>
+  <si>
+    <t>electricity</t>
+  </si>
+  <si>
+    <t>coal</t>
+  </si>
+  <si>
+    <t>natural gas</t>
+  </si>
+  <si>
+    <t>biomass</t>
+  </si>
+  <si>
+    <t>petroleum diesel</t>
+  </si>
+  <si>
+    <t>heat</t>
+  </si>
+  <si>
+    <t>crude oil</t>
+  </si>
+  <si>
+    <t>heavy or residual oil</t>
+  </si>
+  <si>
+    <t>LPG propane or butane</t>
+  </si>
+  <si>
+    <t>hydrogen</t>
+  </si>
+  <si>
     <t>CC Capital Cost of Industrial Energy CCS Equipment</t>
   </si>
   <si>
@@ -104,22 +308,7 @@
     <t>CC Energy Use per Ton Hydrogen Sector CO2 Sequestered</t>
   </si>
   <si>
-    <t>Source:</t>
-  </si>
-  <si>
-    <t>Gaffney Cline</t>
-  </si>
-  <si>
-    <t>National Petroleum Council (NPC) Capture Facility Reference Costs</t>
-  </si>
-  <si>
-    <t>https://www.gaffneycline.com/calculator/npc-scenarios-table</t>
-  </si>
-  <si>
-    <t>Notes:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">This variable captures the capital and O&amp;M costs and energy use of </t>
+    <t>Hydrogen Sector</t>
   </si>
   <si>
     <t>carbon capture and sequestration, for both the industry and hydrogen sectors.</t>
@@ -128,254 +317,59 @@
     <t>It also includes data on energy use per ton CO2 sequestered.</t>
   </si>
   <si>
-    <t>The energy use value here should exclude any energy that is not additional</t>
-  </si>
-  <si>
     <t>to the energy already accounted for in indst/BIFUbC.</t>
   </si>
   <si>
     <t>For example, if a steel mill has excess process heat that</t>
   </si>
   <si>
-    <t>isn't being used, and they use it to power CCS, that heat should be excluded</t>
-  </si>
-  <si>
-    <t>from here, since it does not increase the overall energy demand of the steel</t>
-  </si>
-  <si>
-    <t>mill.</t>
-  </si>
-  <si>
     <t>2020 to 2012 USD</t>
   </si>
   <si>
-    <t>BTU per MWh</t>
-  </si>
-  <si>
-    <t>Low Estimates</t>
-  </si>
-  <si>
-    <t>Facility Type</t>
-  </si>
-  <si>
-    <t>Natural Gas Processing</t>
-  </si>
-  <si>
-    <t>Ethanol Production</t>
-  </si>
-  <si>
-    <t>Ammonia Production</t>
-  </si>
-  <si>
-    <t>Hydrogen Production</t>
-  </si>
-  <si>
-    <t>Cement Plant</t>
-  </si>
-  <si>
-    <t>Refinery Fluidized Catalytic Converter</t>
-  </si>
-  <si>
-    <t>Iron and Steel Plant</t>
-  </si>
-  <si>
-    <t>Industrial Furnace</t>
-  </si>
-  <si>
-    <t>Capacity (tonne / year)</t>
-  </si>
-  <si>
-    <t>Total CapEx (US $ / annual tonne)</t>
-  </si>
-  <si>
-    <t>Electricity usage (MWh / tonne)</t>
-  </si>
-  <si>
-    <t>Gas usage (MWh / tonne)</t>
-  </si>
-  <si>
-    <t>OpEx, Non-energy, annual (% CapEx)</t>
-  </si>
-  <si>
-    <t>Tax rate (%)</t>
-  </si>
-  <si>
-    <t>High Estimates</t>
-  </si>
-  <si>
-    <t>Averages</t>
-  </si>
-  <si>
-    <t>energy pipelines and gas processing 352T353</t>
-  </si>
-  <si>
-    <t>chemicals 20</t>
-  </si>
-  <si>
-    <t>cement and other nonmetallic minerals 239</t>
-  </si>
-  <si>
-    <t>refined petroleum and coke 19</t>
-  </si>
-  <si>
-    <t>iron and steel 241</t>
-  </si>
-  <si>
-    <t>CapEx ($ / annual tonne)</t>
-  </si>
-  <si>
-    <t>Electricity usage (BTU / tonne)</t>
-  </si>
-  <si>
-    <t>Gas usage (BTU / tonne)</t>
-  </si>
-  <si>
-    <t>OpEx, Non-energy</t>
+    <t>electricity if</t>
+  </si>
+  <si>
+    <t>coal if</t>
+  </si>
+  <si>
+    <t>natural gas if</t>
+  </si>
+  <si>
+    <t>biomass if</t>
+  </si>
+  <si>
+    <t>petroleum diesel if</t>
+  </si>
+  <si>
+    <t>heat if</t>
+  </si>
+  <si>
+    <t>crude oil if</t>
+  </si>
+  <si>
+    <t>heavy or residual oil if</t>
+  </si>
+  <si>
+    <t>LPG propane or butane if</t>
+  </si>
+  <si>
+    <t>hydrogen if</t>
+  </si>
+  <si>
+    <t>Energy Use per Ton Sequestered (BTU/gram CO2e)</t>
   </si>
   <si>
     <t>*We use ethanol production as a proxy for the chemicals industry, as we expect ammonia production to be decarbonized via</t>
   </si>
   <si>
     <t>hydrogen electrolysis in our BAU case.</t>
-  </si>
-  <si>
-    <t>Capital cost ($/(metric ton CO2e*yr))</t>
-  </si>
-  <si>
-    <t>agriculture and forestry 01T03</t>
-  </si>
-  <si>
-    <t>coal mining 05</t>
-  </si>
-  <si>
-    <t>oil and gas extraction 06</t>
-  </si>
-  <si>
-    <t>other mining and quarrying 07T08</t>
-  </si>
-  <si>
-    <t>food beverage and tobacco 10T12</t>
-  </si>
-  <si>
-    <t>textiles apparel and leather 13T15</t>
-  </si>
-  <si>
-    <t>wood products 16</t>
-  </si>
-  <si>
-    <t>pulp paper and printing 17T18</t>
-  </si>
-  <si>
-    <t>rubber and plastic products 22</t>
-  </si>
-  <si>
-    <t>glass and glass products 231</t>
-  </si>
-  <si>
-    <t>other metals 242</t>
-  </si>
-  <si>
-    <t>metal products except machinery and vehicles 25</t>
-  </si>
-  <si>
-    <t>computers and electronics 26</t>
-  </si>
-  <si>
-    <t>appliances and electrical equipment 27</t>
-  </si>
-  <si>
-    <t>other machinery 28</t>
-  </si>
-  <si>
-    <t>road vehicles 29</t>
-  </si>
-  <si>
-    <t>nonroad vehicles 30</t>
-  </si>
-  <si>
-    <t>other manufacturing 31T33</t>
-  </si>
-  <si>
-    <t>water and waste 36T39</t>
-  </si>
-  <si>
-    <t>construction 41T43</t>
-  </si>
-  <si>
-    <t>Hydrogen Sector</t>
-  </si>
-  <si>
-    <t>O&amp;M Cost per Ton ($/metric ton CO2e)</t>
-  </si>
-  <si>
-    <t>Energy Use per Ton Sequestered (BTU/gram CO2e)</t>
-  </si>
-  <si>
-    <t>electricity</t>
-  </si>
-  <si>
-    <t>coal</t>
-  </si>
-  <si>
-    <t>natural gas</t>
-  </si>
-  <si>
-    <t>biomass</t>
-  </si>
-  <si>
-    <t>petroleum diesel</t>
-  </si>
-  <si>
-    <t>heat</t>
-  </si>
-  <si>
-    <t>crude oil</t>
-  </si>
-  <si>
-    <t>heavy or residual oil</t>
-  </si>
-  <si>
-    <t>LPG propane or butane</t>
-  </si>
-  <si>
-    <t>hydrogen</t>
-  </si>
-  <si>
-    <t>electricity if</t>
-  </si>
-  <si>
-    <t>coal if</t>
-  </si>
-  <si>
-    <t>natural gas if</t>
-  </si>
-  <si>
-    <t>biomass if</t>
-  </si>
-  <si>
-    <t>petroleum diesel if</t>
-  </si>
-  <si>
-    <t>heat if</t>
-  </si>
-  <si>
-    <t>crude oil if</t>
-  </si>
-  <si>
-    <t>heavy or residual oil if</t>
-  </si>
-  <si>
-    <t>LPG propane or butane if</t>
-  </si>
-  <si>
-    <t>hydrogen if</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -755,143 +749,143 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.28515625" customWidth="1"/>
-    <col min="2" max="2" width="55.85546875" customWidth="1"/>
-    <col min="4" max="4" width="30.5703125" customWidth="1"/>
+    <col min="1" max="1" width="30.26953125" customWidth="1"/>
+    <col min="2" max="2" width="55.81640625" customWidth="1"/>
+    <col min="4" max="4" width="30.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B13" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="2" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="2" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="1"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="1" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="1" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="1" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="B12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="B13" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="A15" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="A16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="1"/>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2">
-      <c r="A25" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="6">
         <v>0.88711067149387013</v>
       </c>
       <c r="B28" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>3412141</v>
       </c>
       <c r="B30" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -906,51 +900,51 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" customWidth="1"/>
-    <col min="2" max="2" width="42.5703125" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7265625" customWidth="1"/>
+    <col min="2" max="2" width="42.54296875" customWidth="1"/>
+    <col min="4" max="4" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="57.95">
+    <row r="1" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A2,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -985,9 +979,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="B3">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A3,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1022,9 +1016,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A4,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1059,9 +1053,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A5,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1096,9 +1090,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A6,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1133,9 +1127,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="B7">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A7,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1170,9 +1164,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="B8">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A8,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1207,9 +1201,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="B9">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A9,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1244,9 +1238,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="B10">
         <f>B9</f>
@@ -1282,9 +1276,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="B11">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A11,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1319,9 +1313,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="B12">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A12,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1356,9 +1350,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="B13">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A13,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1393,9 +1387,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="B14">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A14,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1430,9 +1424,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="B15">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A15,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1467,9 +1461,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="B16">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A16,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1504,9 +1498,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="B17">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A17,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1541,9 +1535,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="B18">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A18,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1578,9 +1572,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="B19">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A19,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1615,9 +1609,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="B20">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A20,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1652,9 +1646,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="B21">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A21,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1689,9 +1683,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="B22">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A22,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1726,9 +1720,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="B23">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A23,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1763,9 +1757,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B24">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A24,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1800,9 +1794,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="B25">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A25,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1837,9 +1831,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="B26">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A26,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -1885,15 +1879,15 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" customWidth="1"/>
-    <col min="2" max="2" width="42.5703125" customWidth="1"/>
+    <col min="1" max="1" width="26.7265625" customWidth="1"/>
+    <col min="2" max="2" width="42.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="29.1">
+    <row r="1" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="B1" s="4" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -1905,83 +1899,83 @@
       <c r="J1" s="7"/>
       <c r="K1" s="7"/>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B2">
         <f>Data!E25/10^12</f>
         <v>6.1418537999999999E-7</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B4">
         <f>Data!E26/10^12</f>
         <v>8.7009595499999985E-6</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="7" t="s">
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
-      <c r="A7" s="7" t="s">
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
-      <c r="A8" s="7" t="s">
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11" s="7" t="s">
         <v>94</v>
-      </c>
-      <c r="B8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
-      <c r="A9" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
-      <c r="A10" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
-      <c r="A11" s="7" t="s">
-        <v>97</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -1996,49 +1990,49 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA25B772-A559-4F07-971A-AC3B6FFE9BE6}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:I30"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+    <col min="1" max="1" width="34.81640625" customWidth="1"/>
     <col min="2" max="9" width="31" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="F3" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="H3" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="I3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B4">
         <v>276216</v>
@@ -2065,9 +2059,9 @@
         <v>259016</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B5">
         <v>16.5</v>
@@ -2094,9 +2088,9 @@
         <v>91.77</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B6">
         <v>0.1</v>
@@ -2123,9 +2117,9 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2152,9 +2146,9 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B8">
         <v>0.06</v>
@@ -2181,9 +2175,9 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B9">
         <v>0.21</v>
@@ -2210,14 +2204,14 @@
         <v>0.21</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="B13" t="str">
         <f>B3</f>
@@ -2252,9 +2246,9 @@
         <v>Industrial Furnace</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B14">
         <f>B4</f>
@@ -2289,9 +2283,9 @@
         <v>259016</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B15">
         <v>27.5</v>
@@ -2318,9 +2312,9 @@
         <v>152.94</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B16">
         <f t="shared" ref="B16:B17" si="2">B6</f>
@@ -2355,9 +2349,9 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B17">
         <f t="shared" si="2"/>
@@ -2392,9 +2386,9 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B18">
         <f t="shared" ref="B18:I18" si="5">B8</f>
@@ -2429,9 +2423,9 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B19">
         <f t="shared" ref="B19:I19" si="6">B9</f>
@@ -2466,30 +2460,30 @@
         <v>0.21</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C22" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="F22" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="G22" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="H22" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B23" t="str">
         <f>B3</f>
         <v>Natural Gas Processing</v>
@@ -2523,7 +2517,7 @@
         <v>Industrial Furnace</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>48</v>
       </c>
@@ -2560,7 +2554,7 @@
         <v>571.58457392593505</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>49</v>
       </c>
@@ -2597,7 +2591,7 @@
         <v>545942.56000000006</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>50</v>
       </c>
@@ -2634,7 +2628,7 @@
         <v>8871566.5999999996</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>51</v>
       </c>
@@ -2671,14 +2665,14 @@
         <v>22.863382957037402</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>53</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -2692,236 +2686,236 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B26"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="44.42578125" customWidth="1"/>
-    <col min="2" max="2" width="24.5703125" customWidth="1"/>
+    <col min="1" max="1" width="44.453125" customWidth="1"/>
+    <col min="2" max="2" width="24.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="29.1">
+    <row r="1" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B1" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="B2" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="B3" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="B4" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="B5" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="B6" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="B7" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="B8" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="B9" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="B10" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A10,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>442.08384092059458</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="B11" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="B12" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="B13" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="B14" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="B15" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="B16" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="B17" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="B18" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="B19" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="B20" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="B21" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="B22" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="B23" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B24" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="B25" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="B26" s="3">
         <f>Data!$I$24*About!$A$28</f>
@@ -2939,236 +2933,236 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B26"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="44.42578125" customWidth="1"/>
-    <col min="2" max="2" width="24.5703125" customWidth="1"/>
+    <col min="1" max="1" width="44.453125" customWidth="1"/>
+    <col min="2" max="2" width="24.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="29.1">
+    <row r="1" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B1" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="B2" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A2,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="B3" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A3,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="B4" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A4,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="B5" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A5,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="B6" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A6,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="B7" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A7,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="B8" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A8,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="B9" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A9,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="B10" s="3">
         <f>Data!$I$24*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="B11" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A11,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>80.122912914199276</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="B12" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A12,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="B13" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A13,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="B14" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A14,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>214.0302346757544</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="B15" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A15,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>157.60743456534033</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="B16" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A16,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="B17" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A17,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="B18" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A18,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="B19" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A19,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="B20" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A20,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="B21" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A21,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="B22" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A22,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="B23" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A23,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B24" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A24,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>85.494272870387022</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="B25" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A25,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
         <v>507.0587751909739</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="B26" s="3">
         <f>IFERROR(INDEX(Data!$24:$24,MATCH('CC-CCoIPCE'!A26,Data!$22:$22,0)),Data!$I$24)*About!$A$28</f>
@@ -3186,96 +3180,96 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B26"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="44.42578125" customWidth="1"/>
-    <col min="2" max="2" width="24.5703125" customWidth="1"/>
+    <col min="1" max="1" width="44.453125" customWidth="1"/>
+    <col min="2" max="2" width="24.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="29.1">
+    <row r="1" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B1" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B2" s="3">
         <f>Data!E24*About!$A$28</f>
         <v>210.77627576977025</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B3" s="3"/>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B4" s="3"/>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B5" s="3"/>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" s="3"/>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B8" s="3"/>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B9" s="3"/>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B10" s="3"/>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B11" s="3"/>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B12" s="3"/>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B13" s="3"/>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B14" s="3"/>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B15" s="3"/>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B16" s="3"/>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" s="3"/>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B18" s="3"/>
     </row>
-    <row r="19" spans="2:2">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B19" s="3"/>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B20" s="3"/>
     </row>
-    <row r="21" spans="2:2">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B21" s="3"/>
     </row>
-    <row r="22" spans="2:2">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B22" s="3"/>
     </row>
-    <row r="23" spans="2:2">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B23" s="3"/>
     </row>
-    <row r="24" spans="2:2">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B24" s="3"/>
     </row>
-    <row r="25" spans="2:2">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B25" s="3"/>
     </row>
-    <row r="26" spans="2:2">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B26" s="3"/>
     </row>
   </sheetData>
@@ -3289,236 +3283,236 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B26"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.140625" customWidth="1"/>
-    <col min="2" max="2" width="25.85546875" customWidth="1"/>
+    <col min="1" max="1" width="19.1796875" customWidth="1"/>
+    <col min="2" max="2" width="25.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="29.1">
+    <row r="1" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B1" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="B3">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="B7">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="B8">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="B9">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="B10">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A10,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>17.683353636823785</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="B11">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="B12">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="B13">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="B14">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="B15">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="B16">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="B17">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="B18">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="B19">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="B20">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="B21">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="B22">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="B23">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B24">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="B25">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="B26">
         <f>Data!$I$27*About!$A$28</f>
@@ -3536,236 +3530,236 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B26"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.140625" customWidth="1"/>
-    <col min="2" max="2" width="25.85546875" customWidth="1"/>
+    <col min="1" max="1" width="19.1796875" customWidth="1"/>
+    <col min="2" max="2" width="25.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="29.1">
+    <row r="1" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B1" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A2,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="B3">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A3,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A4,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A5,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A6,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="B7">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A7,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="B8">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A8,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="B9">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A9,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="B10">
         <f>Data!$I$27*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="B11">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A11,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>5.6086039039939504</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="B12">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A12,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="B13">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A13,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="B14">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A14,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>14.98211642730281</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="B15">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A15,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>7.8803717282670158</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="B16">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A16,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="B17">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A17,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="B18">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A18,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="B19">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A19,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="B20">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A20,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="B21">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A21,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="B22">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A22,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="B23">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A23,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B24">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A24,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>5.1296563722232209</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="B25">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A25,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
         <v>20.282351007638955</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="B26">
         <f>IFERROR(INDEX(Data!$27:$27,MATCH('CC-CCoIPCE'!A26,Data!$22:$22,0)),Data!$I$27)*About!$A$28</f>
@@ -3783,20 +3777,20 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.140625" customWidth="1"/>
-    <col min="2" max="2" width="25.85546875" customWidth="1"/>
+    <col min="1" max="1" width="19.1796875" customWidth="1"/>
+    <col min="2" max="2" width="25.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="29.1">
+    <row r="1" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B1" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B2">
         <f>Data!E27*About!$A$28</f>
@@ -3814,51 +3808,51 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="46.85546875" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="46.81640625" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="57.95">
+    <row r="1" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <f>Data!$I$25/10^12</f>
@@ -3893,9 +3887,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="B3">
         <f>Data!$I$25/10^12</f>
@@ -3930,9 +3924,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <f>Data!$I$25/10^12</f>
@@ -3967,9 +3961,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <f>Data!$I$25/10^12</f>
@@ -4004,9 +3998,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <f>Data!$I$25/10^12</f>
@@ -4041,9 +4035,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="B7">
         <f>Data!$I$25/10^12</f>
@@ -4078,9 +4072,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="B8">
         <f>Data!$I$25/10^12</f>
@@ -4115,9 +4109,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="B9">
         <f>Data!$I$25/10^12</f>
@@ -4152,9 +4146,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="B10">
         <f>IFERROR(INDEX(Data!$25:$25,MATCH('CC-CCoIPCE'!A10,Data!$22:$22,0)),Data!$I$25)*About!$A$28/10^12</f>
@@ -4189,9 +4183,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="B11">
         <f>Data!$I$25/10^12</f>
@@ -4226,9 +4220,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="B12">
         <f>Data!$I$25/10^12</f>
@@ -4263,9 +4257,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="B13">
         <f>Data!$I$25/10^12</f>
@@ -4300,9 +4294,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="B14">
         <f>Data!$I$25/10^12</f>
@@ -4337,9 +4331,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="B15">
         <f>Data!$I$25/10^12</f>
@@ -4374,9 +4368,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="B16">
         <f>Data!$I$25/10^12</f>
@@ -4411,9 +4405,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="B17">
         <f>Data!$I$25/10^12</f>
@@ -4448,9 +4442,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="B18">
         <f>Data!$I$25/10^12</f>
@@ -4485,9 +4479,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="B19">
         <f>Data!$I$25/10^12</f>
@@ -4522,9 +4516,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="B20">
         <f>Data!$I$25/10^12</f>
@@ -4559,9 +4553,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="B21">
         <f>Data!$I$25/10^12</f>
@@ -4596,9 +4590,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="B22">
         <f>Data!$I$25/10^12</f>
@@ -4633,9 +4627,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="B23">
         <f>Data!$I$25/10^12</f>
@@ -4670,9 +4664,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B24">
         <f>Data!$I$25/10^12</f>
@@ -4707,9 +4701,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="B25">
         <f>Data!$I$25/10^12</f>
@@ -4744,9 +4738,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="B26">
         <f>Data!$I$25/10^12</f>
@@ -4784,175 +4778,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
-    <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="79748b23-d81a-423e-9112-21109dc864e6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6FAF0F9-15D0-4CA9-8139-A8DEDD1AC5D2}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{575C02BD-B002-41BB-92FF-55E29ACA380C}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2390A901-A5B0-45DD-9FC2-5ED145B65787}"/>
 </file>
</xml_diff>